<commit_message>
fix export excel phoinhapkho
</commit_message>
<xml_diff>
--- a/dataproduct.api/wwwroot/templates/BM_GiaoNhanPhoiNhapKho.xlsx
+++ b/dataproduct.api/wwwroot/templates/BM_GiaoNhanPhoiNhapKho.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Software\03. ThongKePKH\DATAPRODUCT_V2\dataproduct.api\dataproduct.api\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0973FD09-6DA1-4685-A1CA-870EB0B01462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D319FD10-00B3-48C4-A8D5-A7C15411FB1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BM.12-QT.05.11" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="22">
   <si>
     <t>BM.12/QT.05.11</t>
   </si>
@@ -138,6 +138,9 @@
   </si>
   <si>
     <t>Tình trạng Đúc</t>
+  </si>
+  <si>
+    <t>Tình trạng chốt</t>
   </si>
 </sst>
 </file>
@@ -542,6 +545,12 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -558,12 +567,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1075,7 +1078,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T30"/>
+  <dimension ref="A1:U30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.77734375" style="26" customWidth="1"/>
@@ -1097,7 +1100,7 @@
     <col min="18" max="16384" width="8.88671875" style="26"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1">
+    <row r="1" spans="1:21" s="1" customFormat="1" ht="18.75" customHeight="1">
       <c r="F1" s="2"/>
       <c r="H1" s="3"/>
       <c r="O1" s="2"/>
@@ -1106,7 +1109,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1">
+    <row r="2" spans="1:21" s="1" customFormat="1" ht="18.75" customHeight="1">
       <c r="F2" s="2"/>
       <c r="H2" s="6"/>
       <c r="O2" s="2"/>
@@ -1115,7 +1118,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1">
+    <row r="3" spans="1:21" s="1" customFormat="1" ht="18.75" customHeight="1">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="F3" s="2"/>
@@ -1125,34 +1128,34 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:20" s="1" customFormat="1" ht="9.75" customHeight="1">
+    <row r="4" spans="1:21" s="1" customFormat="1" ht="9.75" customHeight="1">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
     </row>
-    <row r="5" spans="1:20" s="9" customFormat="1" ht="49.5" customHeight="1">
-      <c r="A5" s="34" t="s">
+    <row r="5" spans="1:21" s="9" customFormat="1" ht="49.5" customHeight="1">
+      <c r="A5" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="35"/>
-      <c r="C5" s="35"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="35"/>
-      <c r="G5" s="35"/>
-      <c r="H5" s="35"/>
-      <c r="I5" s="35"/>
-      <c r="J5" s="35"/>
-      <c r="K5" s="35"/>
-      <c r="L5" s="35"/>
-      <c r="M5" s="35"/>
-      <c r="N5" s="35"/>
-      <c r="O5" s="35"/>
-      <c r="P5" s="35"/>
-      <c r="Q5" s="35"/>
-    </row>
-    <row r="6" spans="1:20" s="12" customFormat="1" ht="44.25" customHeight="1">
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="37"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="37"/>
+      <c r="L5" s="37"/>
+      <c r="M5" s="37"/>
+      <c r="N5" s="37"/>
+      <c r="O5" s="37"/>
+      <c r="P5" s="37"/>
+      <c r="Q5" s="37"/>
+    </row>
+    <row r="6" spans="1:21" s="12" customFormat="1" ht="44.25" customHeight="1">
       <c r="A6" s="42" t="s">
         <v>3</v>
       </c>
@@ -1168,41 +1171,44 @@
       <c r="E6" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="39" t="s">
+      <c r="F6" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="38"/>
-      <c r="H6" s="39" t="s">
+      <c r="G6" s="40"/>
+      <c r="H6" s="41" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="38"/>
-      <c r="J6" s="39" t="s">
+      <c r="I6" s="40"/>
+      <c r="J6" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="K6" s="38"/>
-      <c r="L6" s="36" t="s">
+      <c r="K6" s="40"/>
+      <c r="L6" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="M6" s="37"/>
-      <c r="N6" s="38"/>
-      <c r="O6" s="39" t="s">
+      <c r="M6" s="39"/>
+      <c r="N6" s="40"/>
+      <c r="O6" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="P6" s="38"/>
-      <c r="Q6" s="40" t="s">
+      <c r="P6" s="40"/>
+      <c r="Q6" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="R6" s="40" t="s">
+      <c r="R6" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="S6" s="40" t="s">
+      <c r="S6" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="T6" s="40" t="s">
+      <c r="T6" s="34" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:20" s="12" customFormat="1" ht="42" customHeight="1">
+      <c r="U6" s="34" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" s="12" customFormat="1" ht="42" customHeight="1">
       <c r="A7" s="43"/>
       <c r="B7" s="49"/>
       <c r="C7" s="43"/>
@@ -1241,12 +1247,13 @@
       <c r="P7" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="Q7" s="41"/>
-      <c r="R7" s="41"/>
-      <c r="S7" s="41"/>
-      <c r="T7" s="41"/>
-    </row>
-    <row r="8" spans="1:20" s="9" customFormat="1" ht="20.25" customHeight="1">
+      <c r="Q7" s="35"/>
+      <c r="R7" s="35"/>
+      <c r="S7" s="35"/>
+      <c r="T7" s="35"/>
+      <c r="U7" s="35"/>
+    </row>
+    <row r="8" spans="1:21" s="9" customFormat="1" ht="20.25" customHeight="1">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
@@ -1268,7 +1275,7 @@
       <c r="S8" s="16"/>
       <c r="T8" s="16"/>
     </row>
-    <row r="9" spans="1:20" s="9" customFormat="1" ht="20.25" customHeight="1">
+    <row r="9" spans="1:21" s="9" customFormat="1" ht="20.25" customHeight="1">
       <c r="A9" s="15"/>
       <c r="B9" s="15"/>
       <c r="C9" s="17"/>
@@ -1290,7 +1297,7 @@
       <c r="S9" s="18"/>
       <c r="T9" s="18"/>
     </row>
-    <row r="10" spans="1:20" s="9" customFormat="1" ht="20.25" customHeight="1">
+    <row r="10" spans="1:21" s="9" customFormat="1" ht="20.25" customHeight="1">
       <c r="A10" s="15"/>
       <c r="B10" s="15"/>
       <c r="C10" s="17"/>
@@ -1312,7 +1319,7 @@
       <c r="S10" s="18"/>
       <c r="T10" s="18"/>
     </row>
-    <row r="11" spans="1:20" s="9" customFormat="1" ht="20.25" customHeight="1">
+    <row r="11" spans="1:21" s="9" customFormat="1" ht="20.25" customHeight="1">
       <c r="A11" s="15"/>
       <c r="B11" s="15"/>
       <c r="C11" s="17"/>
@@ -1334,7 +1341,7 @@
       <c r="S11" s="18"/>
       <c r="T11" s="18"/>
     </row>
-    <row r="12" spans="1:20" s="9" customFormat="1" ht="20.25" customHeight="1">
+    <row r="12" spans="1:21" s="9" customFormat="1" ht="20.25" customHeight="1">
       <c r="A12" s="15"/>
       <c r="B12" s="15"/>
       <c r="C12" s="17"/>
@@ -1356,7 +1363,7 @@
       <c r="S12" s="18"/>
       <c r="T12" s="18"/>
     </row>
-    <row r="13" spans="1:20" s="9" customFormat="1" ht="20.25" customHeight="1">
+    <row r="13" spans="1:21" s="9" customFormat="1" ht="20.25" customHeight="1">
       <c r="A13" s="15"/>
       <c r="B13" s="15"/>
       <c r="C13" s="17"/>
@@ -1378,7 +1385,7 @@
       <c r="S13" s="18"/>
       <c r="T13" s="18"/>
     </row>
-    <row r="14" spans="1:20" s="9" customFormat="1" ht="20.25" customHeight="1">
+    <row r="14" spans="1:21" s="9" customFormat="1" ht="20.25" customHeight="1">
       <c r="A14" s="28"/>
       <c r="B14" s="28"/>
       <c r="C14" s="29"/>
@@ -1400,7 +1407,7 @@
       <c r="S14" s="30"/>
       <c r="T14" s="30"/>
     </row>
-    <row r="15" spans="1:20" s="11" customFormat="1" ht="22.5" customHeight="1">
+    <row r="15" spans="1:21" s="11" customFormat="1" ht="22.5" customHeight="1">
       <c r="C15" s="20"/>
       <c r="E15" s="21"/>
       <c r="G15" s="10"/>
@@ -1415,7 +1422,7 @@
       <c r="P15" s="23"/>
       <c r="Q15" s="21"/>
     </row>
-    <row r="16" spans="1:20" s="9" customFormat="1" ht="22.5" customHeight="1">
+    <row r="16" spans="1:21" s="9" customFormat="1" ht="22.5" customHeight="1">
       <c r="D16" s="33"/>
       <c r="F16" s="24"/>
       <c r="H16" s="24"/>
@@ -1508,7 +1515,8 @@
       <c r="P30" s="24"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
+    <mergeCell ref="U6:U7"/>
     <mergeCell ref="R6:R7"/>
     <mergeCell ref="S6:S7"/>
     <mergeCell ref="T6:T7"/>
@@ -1537,15 +1545,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
   <Receiver>
@@ -1595,30 +1594,16 @@
 </spe:Receivers>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <WorkflowID xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
-    <DocumentCategory xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb">434;#Tài liệu tham khảo</DocumentCategory>
-    <Required xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
-    <Abstract xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
-    <WorkflowURL xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
-    <Workflow xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
-    <RequestCode xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
-    <DocumentCategoryData xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
-    <DocumentCategoryID xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb">434</DocumentCategoryID>
-    <Index xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
-    <WorkflowStatus xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
-    <_dlc_DocId xmlns="5080075a-a2d0-4f41-835a-c064cb6475b5">CH5WNSYDU3HY-728169239-170</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="5080075a-a2d0-4f41-835a-c064cb6475b5">
-      <Url>https://eoffice.hoaphat.com.vn/record26q2/dungquat/_layouts/15/DocIdRedir.aspx?ID=CH5WNSYDU3HY-728169239-170</Url>
-      <Description>CH5WNSYDU3HY-728169239-170</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100669999A882A93E4F84792C2BAACB93B4" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b80fc736ca040d5fea57e0729c497e52">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5080075a-a2d0-4f41-835a-c064cb6475b5" xmlns:ns3="579933d2-5cc6-4d35-a127-27d5d66984eb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cd04d01efe0e1df8fb7dc4a555e0c373" ns2:_="" ns3:_="">
     <xsd:import namespace="5080075a-a2d0-4f41-835a-c064cb6475b5"/>
@@ -1840,7 +1825,38 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <WorkflowID xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
+    <DocumentCategory xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb">434;#Tài liệu tham khảo</DocumentCategory>
+    <Required xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
+    <Abstract xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
+    <WorkflowURL xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
+    <Workflow xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
+    <RequestCode xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
+    <DocumentCategoryData xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
+    <DocumentCategoryID xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb">434</DocumentCategoryID>
+    <Index xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
+    <WorkflowStatus xmlns="579933d2-5cc6-4d35-a127-27d5d66984eb" xsi:nil="true"/>
+    <_dlc_DocId xmlns="5080075a-a2d0-4f41-835a-c064cb6475b5">CH5WNSYDU3HY-728169239-170</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="5080075a-a2d0-4f41-835a-c064cb6475b5">
+      <Url>https://eoffice.hoaphat.com.vn/record26q2/dungquat/_layouts/15/DocIdRedir.aspx?ID=CH5WNSYDU3HY-728169239-170</Url>
+      <Description>CH5WNSYDU3HY-728169239-170</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{60A291F9-B145-470E-BDD9-891CE98F18C6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F335D64B-1E2A-44D2-9282-9175B2A51B38}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -1848,32 +1864,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{60A291F9-B145-470E-BDD9-891CE98F18C6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1784DC52-2511-4E51-9289-B06AC312985D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="5080075a-a2d0-4f41-835a-c064cb6475b5"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="579933d2-5cc6-4d35-a127-27d5d66984eb"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06D1CE3F-B8AD-4698-9C63-D6EE97198E7F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1890,4 +1881,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1784DC52-2511-4E51-9289-B06AC312985D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="5080075a-a2d0-4f41-835a-c064cb6475b5"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="579933d2-5cc6-4d35-a127-27d5d66984eb"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>